<commit_message>
feat(content): curate 20 real questions from video_1 and video_2
Fill curation JSONs with clean on-screen text (question, options,
faithful explanations, themes, chosen frames) read from the video
frames, then build situation-photo crops + questions.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/questions.xlsx
+++ b/backend/data/questions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,52 +476,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Q001</t>
+          <t>v1q01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>priorités</t>
+          <t>vitesse</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>À cette intersection sans signalisation, qui passe en premier ? (PLACEHOLDER)</t>
+          <t>Le régulateur de vitesse permet de</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Moi</t>
+          <t>Maintenir le véhicule à une vitesse constante</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Le véhicule venant de droite</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Le véhicule venant de gauche</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Personne</t>
-        </is>
-      </c>
+          <t>Bloquer le véhicule à une vitesse maximale</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER : sans signalisation, la priorité est au véhicule venant de la droite.</t>
+          <t>Le régulateur de vitesse permet à la voiture de garder une vitesse constante sans que le conducteur ait à appuyer sur la pédale d'accélérateur. Contrairement au limiteur de vitesse, il ne bloque pas la vitesse du véhicule : même régulateur activé, le conducteur peut accélérer.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>placeholder.png</t>
+          <t>video_1/v1q01.jpg</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -533,52 +525,48 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Q002</t>
+          <t>v1q02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>panneaux</t>
+          <t>cyclistes</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Que signifie ce panneau ? (PLACEHOLDER)</t>
+          <t>Pour limiter le risque d'accident</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Danger</t>
+          <t>Je ralentis</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Interdiction de tourner</t>
+          <t>Je klaxonne</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Obligation de tourner</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Fin d'interdiction</t>
-        </is>
-      </c>
+          <t>Je fais un appel lumineux</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>A,B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>PLACEHOLDER : explication à compléter avec le vrai contenu.</t>
+          <t>Le cycliste arrivant à contre-sens vous a aperçu. Pour limiter le risque d'accident, il suffit de ralentir. Il est inutile de klaxonner ou de faire un appel lumineux.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>placeholder.png</t>
+          <t>video_1/v1q02.jpg</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -590,53 +578,978 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Q003</t>
+          <t>v1q03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>vitesse</t>
+          <t>mécanique-entretien</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Quelle est la vitesse maximale autorisée ici ? (PLACEHOLDER)</t>
+          <t>Je souhaite contrôler mon niveau d'huile. Ce contrôle s'effectue lorsque le moteur est</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>50 km/h</t>
+          <t>Froid</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>80 km/h</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>90 km/h</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>130 km/h</t>
-        </is>
-      </c>
+          <t>Chaud</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pour préserver l'entretien, la fiabilité et la longévité du véhicule, le contrôle des niveaux doit se faire dans des conditions précises : sur sol plat, pour ne pas fausser la mesure, et quelques minutes après avoir coupé le moteur, donc moteur froid, afin d'éviter tout risque de brûlure.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>video_1/v1q03.jpg</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>v1q04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cyclistes</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>La cycliste à gauche</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Circule sur une piste cyclable</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Circule sur une bande cyclable</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Est autorisée à circuler à contre-sens</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>N'est pas autorisée à circuler à contre-sens</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>La cycliste de gauche circule sur une bande cyclable : il n'y a aucune séparation physique entre la zone réservée aux cyclistes et la chaussée, contrairement à une piste cyclable. Elle est autorisée à circuler à contre-sens, comme l'indique la flèche tracée sur la bande cyclable.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>video_1/v1q04.jpg</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>v1q05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>assurance-constat</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Avant d'envoyer mon constat amiable à l'assurance, il m'est possible de modifier les informations</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Au recto : oui</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Au recto : non</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Au verso : oui</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Au verso : non</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Une fois le constat amiable signé par les deux parties, on ne peut modifier que les informations du verso. Le recto contient les informations conjointes, non modifiables, tandis que le verso regroupe les informations personnelles, elles modifiables.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>video_1/v1q05.jpg</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>v1q06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>éclairage-visibilité</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Dans ces conditions, j'allume mes feux</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>De croisement</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>De route</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>De brouillard</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Ici, l'usage des essuie-glaces montre qu'il pleut. En cas de pluie, il faut allumer au minimum les feux de croisement. Les feux de brouillard seraient trop puissants pour cette pluie légère.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>video_1/v1q06.jpg</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>v1q07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>La vitesse sera limitée à 70 km/h</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>À partir du panneau</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Dans 50 m</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Dans 150 m</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Lorsqu'un panneau de limitation de vitesse n'est pas complété par un panonceau de distance, la limitation s'applique dès le panneau.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>video_1/v1q07.jpg</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>v1q08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Je conduis un véhicule prêté. En cas de contrôle, j'ai l'obligation de présenter les papiers du véhicule</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Même si le véhicule que je conduis m'a été prêté, je dois avoir en ma possession les papiers du véhicule. Avant de prendre le volant, il faut donc vérifier que ces documents m'ont bien été confiés.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>video_1/v1q08.jpg</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>v1q09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>distances-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>La distance de sécurité avec le véhicule qui me précède</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Dépend de ma vitesse : oui</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Dépend de ma vitesse : non</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>L'intervalle doit être équivalent à au moins 1 seconde</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>L'intervalle doit être équivalent à au moins 2 secondes</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>La distance de sécurité dépend de la vitesse : plus je roule vite, plus elle doit être importante. L'intervalle avec le véhicule qui me précède doit toujours être d'au moins deux secondes ; j'adapte donc ma distance en fonction de ma vitesse pour respecter cet intervalle.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>video_1/v1q09.jpg</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>v1q10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>équipements-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Le système AFU peut remplacer l'ABS</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER : explication à compléter.</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>none</t>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Le système AFU (aide au freinage d'urgence) amplifie au maximum le freinage du conducteur lors d'un freinage d'urgence. Il ne peut pas remplacer l'ABS (anti-blocage des roues), auquel il est toujours associé ; l'ABS, en revanche, peut équiper un véhicule sans AFU.</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>video_1/v1q10.jpg</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>v2q01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>commandes</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Dans une voiture à boîte manuelle, le frein se trouve sur la pédale</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>De droite</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Du milieu</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>De gauche</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Sur une voiture à boîte manuelle, les trois pédales se répartissent ainsi : à gauche l'embrayage, au milieu le frein et à droite l'accélérateur. Le frein se trouve donc sur la pédale du milieu.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>video_2/v2q01.jpg</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>v2q02</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>priorités</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>À cette intersection, je serai prioritaire sur</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Les véhicules venant de gauche : oui</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Les véhicules venant de gauche : non</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Les véhicules venant de droite : oui</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Les véhicules venant de droite : non</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>À cette intersection, aucun marquage au sol ni panneau n'indique de priorité particulière : j'applique la priorité à droite. Les véhicules venant de ma gauche doivent donc me céder le passage (je suis prioritaire), tandis que je dois céder le passage à ceux venant de ma droite.</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>video_2/v2q02.jpg</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>v2q03</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>permis-à-points</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pour le permis probatoire</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Le capital initial est de 6 points</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Le capital initial est de 12 points</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>En conduite accompagnée et sans commettre d'infraction, j'obtiendrai la totalité de mes points en 2 ans</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>En conduite accompagnée et sans commettre d'infraction, j'obtiendrai la totalité de mes points en 3 ans</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>A,C</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Le capital initial de tout conducteur venant d'obtenir son permis est de 6 points. Pour atteindre les 12 points sans commettre d'infraction, il faut 2 ans en conduite accompagnée et 3 ans en filière traditionnelle.</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>video_2/v2q03.jpg</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>v2q04</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>L'accès sous le pont est interdit aux véhicules</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Mesurant plus de 3,2 mètres de longueur : oui</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Mesurant plus de 3,2 mètres de longueur : non</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Mesurant plus de 3,2 mètres de hauteur : oui</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Mesurant plus de 3,2 mètres de hauteur : non</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Le panneau d'interdiction présent ici interdit l'accès sous le pont aux véhicules de plus de 3,2 m de hauteur : la flèche noire est verticale, elle concerne donc la hauteur. Si les flèches étaient placées sur les côtés, la limitation porterait sur la largeur.</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>video_2/v2q04.jpg</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>v2q05</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sur l'image ci-dessus, ce panneau m'indique un radar</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Fixe</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>La vitesse n'est limitée à 70 km/h qu'au niveau du radar : oui</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>La vitesse n'est limitée à 70 km/h qu'au niveau du radar : non</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Ce panneau de signalisation annonce un radar fixe. La limitation à 70 km/h ne s'applique pas seulement au niveau du radar : je dois continuer à rouler à 70 km/h maximum, même après l'avoir dépassé.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>video_2/v2q05.jpg</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>v2q06</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>écomobilité</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Je souhaite effectuer un petit trajet en ville. Le(s) moyen(s) de transport à privilégier est (sont)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>La marche à pied</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Le vélo</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>La voiture</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>A,B</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Pour un petit trajet en ville, mieux vaut privilégier la marche à pied ou le vélo. Ce comportement réduit la pollution et le trafic : c'est ce qu'on appelle l'écomobilité.</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>video_2/v2q06.jpg</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>v2q07</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Dans cette situation, je peux m'avancer en dépassant le véhicule par la droite</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Vous êtes à un feu rouge avec affectation de voies par direction. Vous pouvez donc avancer dans votre file : ce comportement n'est pas considéré comme un dépassement par la droite.</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>video_2/v2q07.jpg</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>v2q08</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>cyclistes</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Je souhaite continuer tout droit</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Pour dépasser, je dois laisser un intervalle d'au moins 1 m</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Pour dépasser, je dois laisser un intervalle d'au moins 1,5 m</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Dans cette situation, je dépasse</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Dans cette situation, je reste derrière les cyclistes</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>En ville, pour dépasser un deux-roues, je dois laisser un intervalle d'au moins 1 m. Ici, je n'ai pas assez d'espace pour le faire en sécurité : je reste donc derrière les cyclistes en attendant de pouvoir dépasser.</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>video_2/v2q08.jpg</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>v2q09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>premiers-secours</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>La PLS (position latérale de sécurité) se pratique sur une victime</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Qui est consciente : oui</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Qui est consciente : non</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Qui respire : oui</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Qui respire : non</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>La position latérale de sécurité (PLS) se pratique sur une victime inconsciente mais qui respire. Elle permet notamment de ne pas obstruer les voies aériennes et de faciliter l'écoulement des liquides hors de la gorge.</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>video_2/v2q09.jpg</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>v2q10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>distances-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Je circule à 130 km/h</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Ma distance de sécurité est suffisante : oui</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Ma distance de sécurité est suffisante : non</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>À cette vitesse, ma distance d'arrêt est de 90 mètres</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>À cette vitesse, ma distance d'arrêt est de 170 mètres</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>B,D</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>À 130 km/h, l'intervalle de sécurité doit être d'au moins deux traits (bornes d'arrêt d'urgence) : ici la distance est insuffisante, je dois ralentir. Pour estimer la distance d'arrêt, on prend le chiffre des dizaines de la vitesse (13) et on le multiplie par lui-même : 13 × 13 = 169, soit environ 170 m.</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>video_2/v2q10.jpg</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>image</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(content): curate 77 real questions from video_3..video_10
Curate 8 more source videos into the bank (77 questions after dedup),
bringing the total to 97. Read the clean on-screen text from frames,
verify each answer, write faithful French explanations and themes, and
build situation-photo crops + questions.xlsx.

- Reconstructed video_7/video_9 (parser had merged questions) and
  video_10 (English transcript, French on-screen) directly from frames.
- Added DEFAULT_CROPS entries for videos 3-10 (same 1920x632 template).
- Normalized theme accents to a single canonical vocabulary.
- Removed 3 cross-video duplicate questions (v6q09, v8q06, v9q09),
  keeping the richer-option twin of each.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/questions.xlsx
+++ b/backend/data/questions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1002,48 +1002,52 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>v2q01</t>
+          <t>v10q01</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>commandes</t>
+          <t>éclairage-visibilité</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dans une voiture à boîte manuelle, le frein se trouve sur la pédale</t>
+          <t>Dans cette situation, je peux circuler</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>De droite</t>
+          <t>Sans feux</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Du milieu</t>
+          <t>En feux de position seuls</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>De gauche</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>En feux de croisement</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>En feux de route</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B,C</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Sur une voiture à boîte manuelle, les trois pédales se répartissent ainsi : à gauche l'embrayage, au milieu le frein et à droite l'accélérateur. Le frein se trouve donc sur la pédale du milieu.</t>
+          <t>Je circule en agglomération éclairée. Dans ce cas, je peux rouler soit avec les feux de position seuls, soit avec les feux de croisement. Les feux de route sont interdits en agglomération éclairée, et circuler sans aucun feu n'est pas autorisé.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>video_2/v2q01.jpg</t>
+          <t>video_10/v10q01.jpg</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1055,52 +1059,52 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>v2q02</t>
+          <t>v10q02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>priorités</t>
+          <t>mécanique-entretien</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>À cette intersection, je serai prioritaire sur</t>
+          <t>Les caractéristiques des pneumatiques doivent être les mêmes</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Les véhicules venant de gauche : oui</t>
+          <t>Sur les 4 roues : oui</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Les véhicules venant de gauche : non</t>
+          <t>Sur les 4 roues : non</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Les véhicules venant de droite : oui</t>
+          <t>Sur un même essieu : oui</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Les véhicules venant de droite : non</t>
+          <t>Sur un même essieu : non</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>A,D</t>
+          <t>B,C</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>À cette intersection, aucun marquage au sol ni panneau n'indique de priorité particulière : j'applique la priorité à droite. Les véhicules venant de ma gauche doivent donc me céder le passage (je suis prioritaire), tandis que je dois céder le passage à ceux venant de ma droite.</t>
+          <t>La réglementation impose que les caractéristiques des pneumatiques (diamètre, structure, etc.) soient identiques sur un même essieu. En revanche, cette obligation ne s'applique pas à l'ensemble des quatre roues du véhicule.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>video_2/v2q02.jpg</t>
+          <t>video_10/v10q02.jpg</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1112,7 +1116,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>v2q03</t>
+          <t>v10q03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1122,42 +1126,42 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pour le permis probatoire</t>
+          <t>Titulaire du permis B, je peux transporter au maximum</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Le capital initial est de 6 points</t>
+          <t>6 passagers</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Le capital initial est de 12 points</t>
+          <t>8 passagers</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>En conduite accompagnée et sans commettre d'infraction, j'obtiendrai la totalité de mes points en 2 ans</t>
+          <t>10 passagers</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>En conduite accompagnée et sans commettre d'infraction, j'obtiendrai la totalité de mes points en 3 ans</t>
+          <t>12 passagers</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>A,C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Le capital initial de tout conducteur venant d'obtenir son permis est de 6 points. Pour atteindre les 12 points sans commettre d'infraction, il faut 2 ans en conduite accompagnée et 3 ans en filière traditionnelle.</t>
+          <t>Avec un permis B, je peux transporter au maximum 8 passagers, ce qui fait 9 personnes au total en comptant le conducteur. Au-delà de 9 personnes, un permis de transport en commun est nécessaire.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>video_2/v2q03.jpg</t>
+          <t>video_10/v10q03.jpg</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1169,52 +1173,44 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>v2q04</t>
+          <t>v10q04</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>panneaux</t>
+          <t>premiers-secours</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>L'accès sous le pont est interdit aux véhicules</t>
+          <t>Un joint de cannabis s'élimine en</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Mesurant plus de 3,2 mètres de longueur : oui</t>
+          <t>Quelques heures</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Mesurant plus de 3,2 mètres de longueur : non</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Mesurant plus de 3,2 mètres de hauteur : oui</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Mesurant plus de 3,2 mètres de hauteur : non</t>
-        </is>
-      </c>
+          <t>Plusieurs jours</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>B,C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Le panneau d'interdiction présent ici interdit l'accès sous le pont aux véhicules de plus de 3,2 m de hauteur : la flèche noire est verticale, elle concerne donc la hauteur. Si les flèches étaient placées sur les côtés, la limitation porterait sur la largeur.</t>
+          <t>Un joint de cannabis s'élimine en plusieurs jours. L'élimination peut prendre jusqu'à 5 jours dans les urines, voire davantage en cas de consommation régulière.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>video_2/v2q04.jpg</t>
+          <t>video_10/v10q04.jpg</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1226,52 +1222,52 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>v2q05</t>
+          <t>v10q05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>panneaux</t>
+          <t>vitesse</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sur l'image ci-dessus, ce panneau m'indique un radar</t>
+          <t>La visibilité est inférieure à 50 mètres. Je peux rouler au maximum à</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Fixe</t>
+          <t>30 km/h</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>50 km/h</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>La vitesse n'est limitée à 70 km/h qu'au niveau du radar : oui</t>
+          <t>60 km/h</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>La vitesse n'est limitée à 70 km/h qu'au niveau du radar : non</t>
+          <t>70 km/h</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>A,D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Ce panneau de signalisation annonce un radar fixe. La limitation à 70 km/h ne s'applique pas seulement au niveau du radar : je dois continuer à rouler à 70 km/h maximum, même après l'avoir dépassé.</t>
+          <t>Lorsque la visibilité est inférieure à 50 mètres, la vitesse est limitée à 50 km/h maximum. Il s'agit d'une limite : si les conditions l'exigent, je dois rouler encore plus lentement.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>video_2/v2q05.jpg</t>
+          <t>video_10/v10q05.jpg</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1283,48 +1279,44 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>v2q06</t>
+          <t>v10q06</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>écomobilité</t>
+          <t>équipements-de-sécurité</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Je souhaite effectuer un petit trajet en ville. Le(s) moyen(s) de transport à privilégier est (sont)</t>
+          <t>L'utilisation prolongée du régulateur de vitesse peut entraîner une baisse de la vigilance</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>La marche à pied</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Le vélo</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>La voiture</t>
-        </is>
-      </c>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>A,B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Pour un petit trajet en ville, mieux vaut privilégier la marche à pied ou le vélo. Ce comportement réduit la pollution et le trafic : c'est ce qu'on appelle l'écomobilité.</t>
+          <t>L'utilisation prolongée du régulateur de vitesse peut entraîner une baisse de la vigilance, à cause de la monotonie de la conduite : aucune action n'est exercée sur les pédales.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>video_2/v2q06.jpg</t>
+          <t>video_10/v10q06.jpg</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1336,44 +1328,48 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>v2q07</t>
+          <t>v10q07</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>circulation</t>
+          <t>cyclistes</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dans cette situation, je peux m'avancer en dépassant le véhicule par la droite</t>
+          <t>Dans cette situation</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Je fais un appel lumineux</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
+          <t>Je reste dans cette voie</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Je dépasse</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Vous êtes à un feu rouge avec affectation de voies par direction. Vous pouvez donc avancer dans votre file : ce comportement n'est pas considéré comme un dépassement par la droite.</t>
+          <t>Une voiture arrive en sens inverse. Je reste dans ma voie derrière le cycliste. Je pourrai le dépasser une fois que la voiture grise sera passée et que les conditions de sécurité seront réunies.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>video_2/v2q07.jpg</t>
+          <t>video_10/v10q07.jpg</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1385,52 +1381,52 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>v2q08</t>
+          <t>v10q08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>cyclistes</t>
+          <t>écomobilité</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Je souhaite continuer tout droit</t>
+          <t>Les voitures électriques n'émettent</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pour dépasser, je dois laisser un intervalle d'au moins 1 m</t>
+          <t>Aucun polluant : oui</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Pour dépasser, je dois laisser un intervalle d'au moins 1,5 m</t>
+          <t>Aucun polluant : non</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Dans cette situation, je dépasse</t>
+          <t>Aucun gaz à effet de serre : oui</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Dans cette situation, je reste derrière les cyclistes</t>
+          <t>Aucun gaz à effet de serre : non</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>A,D</t>
+          <t>A,C</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>En ville, pour dépasser un deux-roues, je dois laisser un intervalle d'au moins 1 m. Ici, je n'ai pas assez d'espace pour le faire en sécurité : je reste donc derrière les cyclistes en attendant de pouvoir dépasser.</t>
+          <t>En circulation, les voitures électriques n'émettent aucun polluant ni aucun gaz à effet de serre.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>video_2/v2q08.jpg</t>
+          <t>video_10/v10q08.jpg</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1442,52 +1438,52 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>v2q09</t>
+          <t>v10q09</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>premiers-secours</t>
+          <t>signalisation</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>La PLS (position latérale de sécurité) se pratique sur une victime</t>
+          <t>Au feu, je peux</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Qui est consciente : oui</t>
+          <t>Aller tout droit : oui</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Qui est consciente : non</t>
+          <t>Aller tout droit : non</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Qui respire : oui</t>
+          <t>Tourner à droite : oui</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Qui respire : non</t>
+          <t>Tourner à droite : non</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>B,C</t>
+          <t>A,D</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>La position latérale de sécurité (PLS) se pratique sur une victime inconsciente mais qui respire. Elle permet notamment de ne pas obstruer les voies aériennes et de faciliter l'écoulement des liquides hors de la gorge.</t>
+          <t>Le marquage au sol indique que je dois aller tout droit, et un panneau interdit de tourner à droite. Je peux donc aller tout droit mais je ne peux pas tourner à droite.</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>video_2/v2q09.jpg</t>
+          <t>video_10/v10q09.jpg</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1499,55 +1495,4212 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>v10q10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Je suis un jeune conducteur</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Je suis capable de lire tous les indices de conduite en même temps : oui</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Je suis capable de lire tous les indices de conduite en même temps : non</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>L'expérience permet de choisir les indices les plus importants : oui</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>L'expérience permet de choisir les indices les plus importants : non</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>En tant que jeune conducteur, il est difficile de lire de nombreux indices de conduite en même temps : cela vient avec l'expérience. C'est d'ailleurs pour cette raison que les vitesses maximales sont réduites pour les jeunes conducteurs.</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>video_10/v10q10.jpg</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>v2q01</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>commandes</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Dans une voiture à boîte manuelle, le frein se trouve sur la pédale</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>De droite</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Du milieu</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>De gauche</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Sur une voiture à boîte manuelle, les trois pédales se répartissent ainsi : à gauche l'embrayage, au milieu le frein et à droite l'accélérateur. Le frein se trouve donc sur la pédale du milieu.</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>video_2/v2q01.jpg</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>v2q02</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>priorités</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>À cette intersection, je serai prioritaire sur</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Les véhicules venant de gauche : oui</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Les véhicules venant de gauche : non</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Les véhicules venant de droite : oui</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Les véhicules venant de droite : non</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>À cette intersection, aucun marquage au sol ni panneau n'indique de priorité particulière : j'applique la priorité à droite. Les véhicules venant de ma gauche doivent donc me céder le passage (je suis prioritaire), tandis que je dois céder le passage à ceux venant de ma droite.</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>video_2/v2q02.jpg</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>v2q03</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>permis-à-points</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pour le permis probatoire</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Le capital initial est de 6 points</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Le capital initial est de 12 points</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>En conduite accompagnée et sans commettre d'infraction, j'obtiendrai la totalité de mes points en 2 ans</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>En conduite accompagnée et sans commettre d'infraction, j'obtiendrai la totalité de mes points en 3 ans</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>A,C</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Le capital initial de tout conducteur venant d'obtenir son permis est de 6 points. Pour atteindre les 12 points sans commettre d'infraction, il faut 2 ans en conduite accompagnée et 3 ans en filière traditionnelle.</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>video_2/v2q03.jpg</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>v2q04</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>L'accès sous le pont est interdit aux véhicules</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Mesurant plus de 3,2 mètres de longueur : oui</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Mesurant plus de 3,2 mètres de longueur : non</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Mesurant plus de 3,2 mètres de hauteur : oui</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Mesurant plus de 3,2 mètres de hauteur : non</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Le panneau d'interdiction présent ici interdit l'accès sous le pont aux véhicules de plus de 3,2 m de hauteur : la flèche noire est verticale, elle concerne donc la hauteur. Si les flèches étaient placées sur les côtés, la limitation porterait sur la largeur.</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>video_2/v2q04.jpg</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>v2q05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Sur l'image ci-dessus, ce panneau m'indique un radar</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Fixe</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>La vitesse n'est limitée à 70 km/h qu'au niveau du radar : oui</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>La vitesse n'est limitée à 70 km/h qu'au niveau du radar : non</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Ce panneau de signalisation annonce un radar fixe. La limitation à 70 km/h ne s'applique pas seulement au niveau du radar : je dois continuer à rouler à 70 km/h maximum, même après l'avoir dépassé.</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>video_2/v2q05.jpg</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>v2q06</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>écomobilité</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Je souhaite effectuer un petit trajet en ville. Le(s) moyen(s) de transport à privilégier est (sont)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>La marche à pied</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Le vélo</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>La voiture</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>A,B</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Pour un petit trajet en ville, mieux vaut privilégier la marche à pied ou le vélo. Ce comportement réduit la pollution et le trafic : c'est ce qu'on appelle l'écomobilité.</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>video_2/v2q06.jpg</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>v2q07</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Dans cette situation, je peux m'avancer en dépassant le véhicule par la droite</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Vous êtes à un feu rouge avec affectation de voies par direction. Vous pouvez donc avancer dans votre file : ce comportement n'est pas considéré comme un dépassement par la droite.</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>video_2/v2q07.jpg</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>v2q08</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>cyclistes</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Je souhaite continuer tout droit</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Pour dépasser, je dois laisser un intervalle d'au moins 1 m</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Pour dépasser, je dois laisser un intervalle d'au moins 1,5 m</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Dans cette situation, je dépasse</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Dans cette situation, je reste derrière les cyclistes</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>En ville, pour dépasser un deux-roues, je dois laisser un intervalle d'au moins 1 m. Ici, je n'ai pas assez d'espace pour le faire en sécurité : je reste donc derrière les cyclistes en attendant de pouvoir dépasser.</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>video_2/v2q08.jpg</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>v2q09</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>premiers-secours</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>La PLS (position latérale de sécurité) se pratique sur une victime</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Qui est consciente : oui</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Qui est consciente : non</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Qui respire : oui</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Qui respire : non</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>La position latérale de sécurité (PLS) se pratique sur une victime inconsciente mais qui respire. Elle permet notamment de ne pas obstruer les voies aériennes et de faciliter l'écoulement des liquides hors de la gorge.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>video_2/v2q09.jpg</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>v2q10</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>distances-de-sécurité</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Je circule à 130 km/h</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Ma distance de sécurité est suffisante : oui</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Ma distance de sécurité est suffisante : non</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>À cette vitesse, ma distance d'arrêt est de 90 mètres</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>À cette vitesse, ma distance d'arrêt est de 170 mètres</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>B,D</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>À 130 km/h, l'intervalle de sécurité doit être d'au moins deux traits (bornes d'arrêt d'urgence) : ici la distance est insuffisante, je dois ralentir. Pour estimer la distance d'arrêt, on prend le chiffre des dizaines de la vitesse (13) et on le multiplie par lui-même : 13 × 13 = 169, soit environ 170 m.</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>video_2/v2q10.jpg</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>v3q01</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>premiers-secours</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>En cas d'accident, je peux être accusé de non-assistance à personne en danger si</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Je ne porte pas secours aux victimes : oui</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Je ne porte pas secours aux victimes : non</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Je ne fais pas de constat amiable : oui</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Je ne fais pas de constat amiable : non</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Le délit de non-assistance à personne en danger consiste à refuser de porter secours ou d'appeler les secours pour venir en aide à une personne. Ne pas porter secours aux victimes peut donc constituer ce délit. En revanche, ne pas remplir de constat amiable n'est pas un cas de non-assistance. Ce délit expose l'usager à 75 000 euros d'amende et 5 ans d'emprisonnement.</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>video_3/v3q01.jpg</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>v3q02</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>éclairage-visibilité</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Mon rétroviseur intérieur peut posséder une position nuit pour atténuer l'éblouissement engendré par une voiture qui me suit</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Un rétroviseur intérieur possède très souvent une position nuit permettant de réduire l'éblouissement provoqué par les phares d'un véhicule qui suit. Cette position peut être activée manuellement par le conducteur ou, sur les voitures plus modernes, de façon automatique. On parle alors de rétroviseur électrochrome.</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>video_3/v3q02.jpg</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>v3q03</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Je roule à 90 km/h, je suis bien placé</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Comme l'indique le marquage au sol, avec des traits larges et rapprochés, la voie de droite est une voie réservée aux véhicules lents. Seuls les véhicules roulant à moins de 60 km/h doivent y circuler. Roulant à 90 km/h, je suis donc bien placé sur la voie de gauche.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>video_3/v3q03.jpg</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>v3q04</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Ces panneaux m'indiquent</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Un stationnement limité par disque : oui</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Un stationnement limité par disque : non</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Une priorité à droite : oui</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Une priorité à droite : non</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Le panneau d'indication signale un stationnement payant, et non un stationnement limité par disque, comme le montre la présence d'un horodateur sur le panneau. Le panneau de danger, quant à lui, annonce bien une priorité à droite.</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>video_3/v3q04.jpg</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>v3q05</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>commandes</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Ces commandes permettent de contrôler</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Le limiteur de vitesse</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Le régulateur de vitesse</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>L'autoradio</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Le système ABS</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>A,B</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Ces commandes situées sur le volant permettent de contrôler le régulateur et le limiteur de vitesse. On distingue en effet les signes plus et moins qui servent à régler la vitesse souhaitée.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>video_3/v3q05.jpg</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>v3q06</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Je souhaite aller à Sénart</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Je me place immédiatement sur la voie de gauche</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Je suis bien placé</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Je continue tout droit</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Pour aller à Sénart, il aurait fallu se placer sur la voie de gauche. Dans cette situation, il est désormais trop tard pour changer de voie sans risque : je continue donc tout droit dans ma voie.</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>video_3/v3q06.jpg</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>v3q07</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>éclairage-visibilité</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>La circulation ralentit fortement devant moi et je suis le dernier véhicule de ma file. J'allume mes feux de détresse</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Lorsque la circulation ralentit fortement devant vous, vous devez allumer vos feux de détresse si vous êtes le dernier véhicule de votre file. Ce comportement permet d'avertir les usagers qui arrivent derrière vous.</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>video_3/v3q07.jpg</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>v3q08</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>premiers-secours</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Une consommation d'alcool excessive</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Diminue le temps de réaction</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Augmente le temps de réaction</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Multiplie le risque d'accident</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Une consommation d'alcool excessive multiplie le risque d'accident et augmente le temps de réaction du conducteur, qui met alors plus de temps à agir face à une situation à risque. Attention au piège : le temps de réaction ne diminue pas, il augmente.</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>video_3/v3q08.jpg</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>v3q09</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>permis-à-points</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Conduire avec un téléphone à la main, sans commettre une autre infraction, entraine</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Une amende</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Un retrait de 3 points</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Une suspension de permis</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>A,B</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Téléphoner avec le téléphone à la main représente un fort risque au volant. Ce comportement est interdit et entraîne une amende ainsi qu'un retrait de 3 points sur le permis de conduire. La suspension du permis n'intervient que si le conducteur commet en même temps une autre infraction.</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>video_3/v3q09.jpg</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>v3q10</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Dans cette situation</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Je vais entrer sur une autoroute</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Je vais entrer sur une route à accès réglementé</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Je pourrais y rencontrer des véhicules agricoles : oui</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Je pourrais y rencontrer des véhicules agricoles : non</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>B,D</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Le panneau de signalisation aperçu sur la droite indique que je vais entrer sur une route à accès réglementé, et non sur une autoroute. Comme pour les autoroutes, une route à accès réglementé est interdite aux véhicules lents, tels que les véhicules agricoles.</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>video_3/v3q10.jpg</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>v4q01</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>distances-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Je circule à 50 km/h. La distance d'arrêt de mon véhicule est de</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>15 mètres</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>25 mètres</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>30 mètres</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>50 mètres</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Pour calculer la distance d'arrêt, on multiplie par lui-même le chiffre des dizaines de la vitesse. À 50 km/h, cela donne 5 × 5 = 25 mètres. À titre de comparaison, à 110 km/h la distance d'arrêt serait de 11 × 11 = 121 mètres.</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>video_4/v4q01.jpg</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>v4q02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>distances-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Je circule à 50 km/h. La distance de sécurité à laisser avec le véhicule qui me précède doit être d'au moins</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>30 mètres</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>40 mètres</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>50 mètres</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>60 mètres</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Pour calculer la distance de sécurité à laisser avec le véhicule qui précède, on multiplie par 6 le chiffre des dizaines de la vitesse. À 50 km/h, la distance minimale est donc de 5 × 6 = 30 mètres. Pour la retenir : le mot « sécurité » commence par un S, comme le chiffre 6.</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>video_4/v4q02.jpg</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>v4q03</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>distances-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Je circule à 90 km/h, la distance que parcourt mon véhicule en 1 seconde est de</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>7 mètres</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>17 mètres</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>27 mètres</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>37 mètres</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Pour calculer la distance parcourue par un véhicule en une seconde, on multiplie par 3 le chiffre des dizaines de la vitesse. À 90 km/h, cela donne 9 × 3 = 27 mètres en une seconde. À 50 km/h, ce serait 5 × 3 = 15 mètres.</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>video_4/v4q03.jpg</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>v4q04</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>distances-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>L'intervalle de temps à laisser entre mon véhicule et celui qui me précède doit être au minimum de</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>1 seconde</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2 secondes</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>3 secondes</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>4 secondes</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>L'intervalle de temps à laisser avec le véhicule qui précède doit être d'au moins 2 secondes. Pour le vérifier, choisissez un repère fixe au niveau du véhicule qui vous précède, par exemple un arbre, puis prononcez « un éléphant, deux éléphants » : vous ne devez atteindre ce repère qu'après cette phrase, pas avant.</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>video_4/v4q04.jpg</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>v4q05</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>L'alcoolémie maximale à ne pas dépasser pour un jeune conducteur est de</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>0,1 g/L de sang</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>0,2 g/L de sang</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>0,4 g/L de sang</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0,5 g/L de sang</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>L'alcoolémie maximale à ne pas dépasser pour un jeune conducteur (en permis probatoire) est de 0,2 g/L de sang, soit 0,1 mg d'alcool pur par litre d'air expiré. Pour passer des grammes par litre de sang aux milligrammes par litre d'air expiré, il suffit de diviser la valeur par deux.</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>video_4/v4q05.jpg</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>v4q06</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>L'alcoolémie maximale à ne pas dépasser pour un conducteur expérimenté est de</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>0,2 g/L de sang</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>0,3 g/L de sang</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>0,4 g/L de sang</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>0,5 g/L de sang</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>L'alcoolémie maximale à ne pas dépasser pour un conducteur expérimenté est de 0,5 g/L de sang, soit 0,25 mg d'alcool pur par litre d'air expiré.</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>video_4/v4q06.jpg</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>v4q07</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>équipements-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Pour signaler une panne ou un accident, le triangle de présignalisation doit être posé en amont du véhicule à au moins</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>10 mètres</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>30 mètres</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>50 mètres</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>100 mètres</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Le triangle de présignalisation doit être placé à une distance d'au moins 30 mètres en amont de la panne ou de l'accident. Pour des raisons de sécurité, il est en revanche vivement déconseillé de le placer sur une autoroute.</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>video_4/v4q07.jpg</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>v4q08</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>premiers-secours</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Suite à un accident de la route, un conducteur peut joindre les services de secours en composant le</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>A,B,D</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Selon la nature de l'accident, on peut contacter les services de secours en composant le 15 pour le SAMU, le 18 pour les pompiers, ou le 112, numéro d'urgence valable dans toute l'Union européenne.</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>video_4/v4q08.jpg</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>v4q09</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>distances-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>La distance latérale de sécurité à laisser avec un usager vulnérable doit être d'au moins</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>En ville : 1 mètre</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>En ville : 1,5 mètre</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Hors agglomération : 1 mètre</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Hors agglomération : 1,5 mètre</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Lorsqu'on dépasse un usager vulnérable, la distance latérale de sécurité doit être d'au moins 1 mètre en ville et d'au moins 1,5 mètre hors agglomération. À retenir : en ville, il y a souvent moins de place pour dépasser, on tolère donc 1 mètre au lieu de 1,5 mètre.</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>video_4/v4q09.jpg</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>v4q10</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>équipements-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Un enfant est autorisé à s'installer à l'avant de la voiture à partir de</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>5 ans</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>7 ans</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>10 ans</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>12 ans</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Le code de la route autorise un enfant à s'installer à l'avant de la voiture à partir de 10 ans. Par ailleurs, les enfants de moins de 135 cm doivent être transportés dans un siège homologué, adapté à leur poids et à leur taille.</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>video_4/v4q10.jpg</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>v5q01</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>signalisation</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Dans 400 mètres, au péage, je pourrai payer</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>En carte restaurant</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>En espèces</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>En carte bancaire</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Avec un télépéage</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>B,C,D</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Le panneau situé sur la droite annonce le péage et indique les moyens de paiement acceptés. On peut y régler avec un télépéage, une carte bancaire ou en espèces. Le paiement en carte restaurant n'est en revanche pas prévu.</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>video_5/v5q01.jpg</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>v5q02</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>vitesse</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Je circule à 130 km/h, j'arriverai à Blois dans environ</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>15 minutes</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>30 minutes</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Le panneau indique que Blois se situe à environ 62 km. À 130 km/h, je parcours 130 km en une heure ; il me faut donc à peu près la moitié de ce temps pour couvrir un peu moins de la moitié de cette distance, soit environ 30 minutes.</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>video_5/v5q02.jpg</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>v5q03</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>priorités</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Le véhicule gris souhaite tourner à droite</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Je lui cède le passage</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Je continue</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Le véhicule gris souhaite tourner à droite, mais le marquage au sol montre qu'il n'est pas prioritaire. Je bénéficie donc de la priorité de passage et je peux continuer ma route.</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>video_5/v5q03.jpg</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>v5q04</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>mécanique-entretien</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Aucune contrainte (dimensions, couleur, marque...) n'existe pour le remplacement d'un pneumatique</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>C'est faux : lors du remplacement d'un pneumatique, de nombreux critères doivent être respectés, comme la largeur, la hauteur ou le diamètre du pneu. Ces informations sont généralement indiquées sur le flanc du pneumatique.</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>video_5/v5q04.jpg</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>v5q05</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>commandes</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Je souhaite me garer à droite</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Le stationnement se fait en bataille</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Le stationnement se fait en créneau</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Je dois me garer en marche avant</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Je dois me garer en marche arrière</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>B,D</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Les voitures stationnées à droite sont parallèles au trottoir : il s'agit donc d'un stationnement en créneau. Pour m'y garer, je dois effectuer ma manœuvre en marche arrière.</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>video_5/v5q05.jpg</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>v5q06</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>équipements-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Je suis dans un véhicule ne possédant pas de place à l'arrière. Je peux placer mon enfant de moins de 10 ans à l'avant</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>En principe, un enfant de moins de 10 ans doit être installé à l'arrière du véhicule. Cependant, si le véhicule ne possède pas de banquette arrière, l'enfant peut exceptionnellement prendre place à l'avant.</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>video_5/v5q06.jpg</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>v5q07</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>permis-à-points</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Mon permis de conduire vient d'être invalidé. Je peux suivre un stage de sensibilisation pour regagner mes points</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>C'est faux : lorsque le permis est invalidé, il n'est plus possible de récupérer des points en suivant un stage de sensibilisation. Le stage ne permet de récupérer des points que sur un permis encore valide.</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>video_5/v5q07.jpg</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>v5q08</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>mécanique-entretien</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Mon véhicule Diesel indique un régime moteur à 3500 tours/minute</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Je rétrograde à la vitesse inférieure</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Je conserve mon rapport de vitesse</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Je passe la vitesse supérieure</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Le régime d'un moteur Diesel doit rester autour de 1500 tours/minute. À 3500 tours/minute, le régime est trop élevé : je dois passer la vitesse supérieure pour réduire le nombre de tours par minute et adopter une conduite plus économique.</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>video_5/v5q08.jpg</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>v5q09</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>premiers-secours</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Pour éviter la somnolence, je peux</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Augmenter le son de l'autoradio : oui</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Augmenter le son de l'autoradio : non</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Ouvrir la vitre pour faire entrer l'air : oui</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Ouvrir la vitre pour faire entrer l'air : non</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>B,D</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Augmenter le son de l'autoradio ou ouvrir la vitre ne sont pas des moyens efficaces pour lutter contre la somnolence. Le seul remède réellement efficace est de faire une pause : il faut s'arrêter au moins 15 minutes toutes les deux heures de conduite.</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>video_5/v5q09.jpg</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>v5q10</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>assurance-constat</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Je viens d'acheter un véhicule</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Mon véhicule doit obligatoirement être assuré : oui</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Mon véhicule doit obligatoirement être assuré : non</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>L'assurance à "Responsabilité Civile" est le minimum obligatoire : oui</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>L'assurance à "Responsabilité Civile" est le minimum obligatoire : non</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>A,C</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Après l'achat d'un véhicule, celui-ci doit obligatoirement être assuré pour pouvoir circuler. Le minimum obligatoire est l'assurance à responsabilité civile, dite "au tiers", qui couvre les dommages causés aux autres usagers impliqués dans un accident.</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>video_5/v5q10.jpg</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>v6q01</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>équipements-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>L'éthylotest fait partie des éléments obligatoires à avoir dans la voiture</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Non. Depuis mai 2020, l'éthylotest ne fait plus partie des éléments obligatoires à avoir dans son véhicule. Vous ne risquez donc aucune sanction si vous n'en possédez pas.</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>video_6/v6q01.jpg</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>v6q02</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Ayant oublié d'effectuer mon contrôle technique dans les temps, je risque</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Une amende</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Une perte de points</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Une invalidation de mon permis de conduire</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Si la date de validité de votre contrôle technique est dépassée, vous risquez une amende de 135 euros et une éventuelle immobilisation du véhicule. Il n'y a en revanche ni perte de points, ni invalidation du permis.</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>video_6/v6q02.jpg</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>v6q03</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>permis-à-points</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>La perte de tous les points sur le permis de conduire entraîne</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Une suspension du permis</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Une invalidation du permis</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Attention à ne pas confondre ces deux termes. Lorsqu'il ne reste plus aucun point, le permis est invalidé : la conduite est interdite. L'invalidation s'applique à toutes les catégories : si vous possédez aussi un permis moto ou poids lourd, ceux-ci sont également invalidés.</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>video_6/v6q03.jpg</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>v6q04</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Je suis bien positionné</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Pour aller à gauche : oui</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Pour aller à gauche : non</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Pour aller tout droit : oui</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Pour aller tout droit : non</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Le marquage au sol indique que je suis dans la bonne voie pour aller tout droit. En revanche, si je souhaite tourner à gauche, je ne suis pas bien placé et je dois changer de voie.</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>video_6/v6q04.jpg</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>v6q05</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Je circule sur</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Une départementale</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Une nationale</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Une autoroute</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Le panneau à fond bleu situé sur la droite indique que je circule sur une autoroute. Il annonce ici la prochaine aire d'autoroute, à 300 mètres.</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>video_6/v6q05.jpg</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>v6q06</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>vitesse</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Les chances de survie d'un piéton percuté à 50 km/h sont de</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>20 %</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>70 %</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Un piéton percuté à 50 km/h n'a que 20 % de chances de survie. En ville, il faut donc faire particulièrement attention aux usagers vulnérables.</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>video_6/v6q06.jpg</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>v6q07</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>éclairage-visibilité</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>La nuit, un véhicule seul en agglomération non éclairée doit utiliser ses feux</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>De brouillard avant</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>De croisement</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>De route</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>La nuit, dans une agglomération non éclairée et en l'absence d'autres usagers, le véhicule doit utiliser ses feux de route. Pensez cependant à repasser en feux de croisement dès que vous croisez un autre usager.</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>video_6/v6q07.jpg</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>v6q08</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>priorités</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Dans cette situation</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>En cas d'embouteillage, je peux rouler sur la voie la plus à droite : oui</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>En cas d'embouteillage, je peux rouler sur la voie la plus à droite : non</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Je reste sur ma voie et je tourne à droite au feu. Je dois laisser la priorité aux usagers roulant sur la voie la plus à droite : oui</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Je reste sur ma voie et je tourne à droite au feu. Je dois laisser la priorité aux usagers roulant sur la voie la plus à droite : non</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>La voie la plus à droite est une voie de bus : je ne peux pas y rouler, même en cas d'embouteillage. Si je tourne à droite au feu, je dois rester attentif aux usagers qui l'empruntent et leur laisser la priorité, car je ne suis pas prioritaire sur eux.</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>video_6/v6q08.jpg</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>v6q10</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Il n'y a plus de place disponible pour stationner à gauche. Je peux stationner sur le trottoir de droite</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Non. Aucune signalisation n'autorise le stationnement sur le trottoir de droite : je ne peux donc pas m'y garer. En stationnant ici, je gênerais le passage réservé à la circulation des piétons.</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>video_6/v6q10.jpg</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>v7q01</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>vitesse</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Le premier facteur d'accident mortel au volant est</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>L'alcool</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>La drogue</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>La vitesse</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Le premier facteur d'accident mortel au volant en France est la vitesse. Elle allonge la distance de freinage et aggrave la violence des chocs.</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>video_7/v7q01.jpg</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>v7q02</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Un panneau de fin d'interdiction peut mettre fin à</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Une limitation de vitesse</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Une interdiction de stationner</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Une interdiction de dépasser</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>A,C</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Le panneau de fin d'interdiction met fin à toutes les interdictions signalées précédemment pour un véhicule en mouvement. Il peut donc lever une limitation de vitesse ou une interdiction de dépasser, mais pas une interdiction de stationner, car un véhicule stationné est à l'arrêt et non en mouvement.</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>video_7/v7q02.jpg</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>v7q03</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>écomobilité</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Une allure constante permet d'éviter une surconsommation de carburant</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Rouler à une allure constante permet d'éviter la surconsommation de carburant. C'est en roulant à une vitesse irrégulière, avec des accélérations et des freinages répétés, que l'on consomme le plus.</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>video_7/v7q03.jpg</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>v7q04</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>éclairage-visibilité</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>L'éblouissement perturbe la vision du conducteur</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Environ 1 seconde</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Environ 5 secondes</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>L'éblouissement est un phénomène dangereux car il perturbe la vision du conducteur pendant environ 5 secondes. Durant ce laps de temps, le conducteur ne perçoit plus toutes les informations et son temps de réaction est allongé.</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>video_7/v7q04.jpg</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>v7q05</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>commandes</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Le régulateur de vitesse est adapté pour une conduite</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>En ville : oui</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>En ville : non</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Sur autoroute : oui</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Sur autoroute : non</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>En ville, l'utilisation du régulateur de vitesse n'est pas adaptée car il faut sans cesse ajuster sa vitesse à cause des nombreuses intersections, feux rouges et ronds-points. Le régulateur est en revanche bien adapté sur autoroute, où l'allure reste stable.</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>video_7/v7q05.jpg</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>v7q06</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>La MMTA (anciennement PTAC) de ma remorque est de 600 kg</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Le permis B est suffisant : oui</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Le permis B est suffisant : non</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>La remorque doit avoir sa propre plaque d'immatriculation : oui</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>La remorque doit avoir sa propre plaque d'immatriculation : non</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>A,C</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>La MMTA (masse maximale techniquement admissible) remplace l'ancien terme PTAC. Le permis B suffit pour tracter une remorque jusqu'à 750 kg, donc il est suffisant ici. De plus, dès que la MMTA dépasse 500 kg, la remorque doit posséder sa propre carte grise et sa propre plaque d'immatriculation.</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>video_7/v7q06.jpg</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>v7q07</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>premiers-secours</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Si je suis témoin d'un accident, je dois (dans l'ordre)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Secourir, Protéger, Alerter</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Protéger, Alerter, Secourir</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Secourir, Alerter, Protéger</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Alerter, Protéger, Secourir</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Face à un accident, la conduite à tenir dans l'ordre est : protéger la zone de l'accident et les victimes, alerter les secours, puis secourir la victime. La séquence correcte est donc Protéger, Alerter, Secourir.</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>video_7/v7q07.jpg</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>v7q08</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Ce panneau indique</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>L'entrée dans une zone de rencontre : oui</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>L'entrée dans une zone de rencontre : non</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Je pourrais y rencontrer : des voitures</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Je pourrais y rencontrer : des cyclistes</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>A,C,D</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Ce panneau signale l'entrée dans une zone de rencontre, où la vitesse est limitée à 20 km/h. On peut notamment y croiser des voitures et des cyclistes. Attention : une même sous-question peut comporter deux bonnes réponses.</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>video_7/v7q08.jpg</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>v7q09</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>assurance-constat</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>À jeun, le pic d'alcoolémie est atteint après environ</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>30 minutes</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>1 heure</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>2 heures</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>À jeun, le pic d'alcoolémie est atteint après environ 30 minutes. Ce délai passe à environ une heure si l'on a mangé avant de consommer de l'alcool.</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>video_7/v7q09.jpg</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>v7q10</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Sur une place de livraison partagée, je peux</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>M'arrêter</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Stationner sous certaines conditions</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Stationner tout le temps</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>A,B</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Sur une place de livraison partagée, il est possible de s'arrêter. On peut également y stationner, mais seulement sous certaines conditions, par exemple les jours fériés et le dimanche.</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>video_7/v7q10.jpg</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>v8q01</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>mécanique-entretien</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Sur un même essieu, la différence d'usure entre deux pneumatiques ne doit pas dépasser</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>1 mm</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>5 mm</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>15 mm</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Sur un même essieu, la différence d'usure entre les deux pneumatiques ne doit pas dépasser 5 mm. Un écart plus important pourrait entraîner un mauvais contact des pneus avec la route et compromettre la tenue de route.</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>video_8/v8q01.jpg</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>v8q02</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Le véhicule de gauche roule moins vite que moi</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Je ralentis</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Je conserve mon allure</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>J'accélère</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Le véhicule de gauche roule moins vite que moi. Si je ne ralentis pas, je vais le dépasser par la droite, ce qui n'est pas autorisé. Je dois donc ralentir et me placer derrière lui pour le dépasser par la gauche.</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>video_8/v8q02.jpg</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>v8q03</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>signalisation</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Le feu est orange clignotant</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Je m'arrête</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Je ralentis et je passe</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Un feu orange clignotant n'oblige pas à s'arrêter : il signale une intersection ou un passage nécessitant une vigilance particulière. Je ralentis, je redouble d'attention et je passe.</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>video_8/v8q03.jpg</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>v8q04</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Dans cette situation</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Je ralentis</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Je maintiens l'allure</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>J'accélère</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Des piétons sont présents sur le côté droit et créent une zone d'incertitude. Je dois ralentir et faire particulièrement attention, car l'un d'eux pourrait s'engager sur la chaussée.</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>video_8/v8q04.jpg</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>v8q05</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>éclairage-visibilité</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Les feux de croisement éclairent</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Plus loin à droite qu'à gauche</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Plus loin à gauche qu'à droite</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>À la même distance à droite et à gauche</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Les feux de croisement gauche et droit n'éclairent pas à la même distance. Pour ne pas éblouir les usagers arrivant en face, le feu de croisement gauche éclaire moins loin que le droit : ils éclairent donc plus loin à droite qu'à gauche.</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>video_8/v8q05.jpg</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>v8q07</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>premiers-secours</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Laisser seul un enfant au soleil dans une voiture est un comportement très dangereux</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Un enfant laissé seul dans une voiture au soleil risque de suffoquer et de se déshydrater très rapidement, la température montant très vite dans l'habitacle. Même s'il dort, il faut le réveiller et ne jamais le laisser seul.</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>video_8/v8q07.jpg</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>v8q08</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>La voiture devant moi a enclenché ses feux de détresse. Je peux dépasser</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Les feux de détresse signalent que le véhicule est à l'arrêt ou en difficulté. Aucun usager n'arrivant en face, je suis autorisé à le dépasser : je mets mon clignotant et je le dépasse en restant très prudent.</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>video_8/v8q08.jpg</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>v8q09</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>premiers-secours</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Je suis témoin d'un accident ayant entraîné des dommages corporels</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>En cas de danger immédiat, je peux déplacer la victime : oui</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>En cas de danger immédiat, je peux déplacer la victime : non</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Je peux donner à boire à la victime : oui</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Je peux donner à boire à la victime : non</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Lors d'un accident corporel, il est recommandé de ne pas déplacer la victime, sauf en cas de danger immédiat où l'on peut alors la mettre à l'abri. Il ne faut jamais lui donner à boire, car cela pourrait compromettre une éventuelle opération médicale.</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>video_8/v8q09.jpg</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>v8q10</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>mécanique-entretien</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Le niveau sonore de mon véhicule</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Peut être contrôlé par les forces de l'ordre : oui</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Peut être contrôlé par les forces de l'ordre : non</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Peut être mesuré près du moteur</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Peut être mesuré à la sortie du pot d'échappement</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Le niveau sonore d'un véhicule peut être contrôlé par les forces de l'ordre, à l'aide d'un dispositif placé à la sortie du pot d'échappement. Pour être en conformité avec la réglementation, il ne doit pas dépasser la limite fixée en décibels.</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>video_8/v8q10.jpg</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>v9q01</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>équipements-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Je risque une amende</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Si mon enfant n'est pas installé dans un siège adapté à sa corpulence : oui</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Si mon enfant n'est pas installé dans un siège adapté à sa corpulence : non</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Si je n'ai pas activé la sécurité enfant : oui</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Si je n'ai pas activé la sécurité enfant : non</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>A,D</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Je risque effectivement une amende si mon enfant n'est pas installé dans un siège homologué et adapté à son poids et à sa taille. En revanche, la sécurité enfant n'est pas un dispositif obligatoire : ne pas l'avoir activée n'expose à aucune amende.</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>video_9/v9q01.jpg</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>v9q02</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>équipements-de-sécurité</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Mes passagers n'ont pas attaché leur ceinture de sécurité. Je risque une amende</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Pour le passager majeur : oui</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Pour le passager majeur : non</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Pour le passager mineur : oui</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Pour le passager mineur : non</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>En tant que conducteur, je dois m'assurer que tous les passagers ont bien attaché leur ceinture avant de partir. Cependant, je ne risque une amende que pour un passager mineur non attaché. Un passager majeur non attaché devra s'acquitter lui-même de sa propre amende.</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>video_9/v9q02.jpg</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>v9q03</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>premiers-secours</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>La consommation d'alcool</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Augmente les effets de l'éblouissement : oui</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Augmente les effets de l'éblouissement : non</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Rétrécit le champ visuel du conducteur : oui</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Rétrécit le champ visuel du conducteur : non</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>A,C</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>La consommation d'alcool a plusieurs effets néfastes sur la conduite. Parmi eux, on retrouve l'augmentation des effets de l'éblouissement et la diminution (le rétrécissement) du champ visuel du conducteur.</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>video_9/v9q03.jpg</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>v9q04</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>signalisation</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Pour signaler un ralentissement aux usagers qui me suivent, je peux</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Faire un appel de phare</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Appuyer par intermittence sur la pédale de frein</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Klaxonner</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Pour signaler un ralentissement aux usagers qui me suivent, je peux appuyer légèrement et par intermittence sur la pédale de frein. Cela allume mes feux stop de façon discontinue et attire ainsi l'attention du conducteur qui me suit.</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>video_9/v9q04.jpg</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>v9q05</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>éclairage-visibilité</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Dans ce tunnel, j'allume mes feux</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>De croisement</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>De route</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Dans ce tunnel éclairé, je dois obligatoirement allumer mes feux de croisement. Les feux de route sont réservés aux situations où la chaussée n'est pas éclairée, hors agglomération.</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>video_9/v9q05.jpg</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>v9q06</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>permis-à-points</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Durant ma période probatoire, j'ai commis une infraction entrainant un retrait de 3 points. Je dois obligatoirement suivre un stage de sensibilisation à la sécurité routière</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Le stage de sensibilisation à la sécurité routière est obligatoire pour tout retrait de points supérieur ou égal à 3 durant la période probatoire. Je dois donc suivre ce stage.</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>video_9/v9q06.jpg</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>v9q07</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>documents</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>À la vente du véhicule, le contrôle technique doit dater au maximum de</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>3 mois</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>6 mois</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>8 mois</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>1 an</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Lors de la vente d'un véhicule, le contrôle technique doit être fourni par le vendeur et dater de moins de 6 mois.</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>video_9/v9q07.jpg</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>v9q08</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>circulation</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Dans cette situation</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Je dépasse</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Je reste derrière le bus</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Le bus est en train de quitter son arrêt : il a activé son clignotant gauche. Je lui facilite le passage en restant derrière lui. De plus, la visibilité est trop mauvaise pour dépasser en sécurité.</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>video_9/v9q08.jpg</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>v9q10</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>panneaux</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Dans cette rue</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Je pourrais croiser des véhicules venant en sens inverse : oui</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Je pourrais croiser des véhicules venant en sens inverse : non</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Je pourrais croiser des vélos venant en sens inverse : oui</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Je pourrais croiser des vélos venant en sens inverse : non</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>B,C</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Le panneau carré bleu indique une voie à double sens dont le sens opposé est réservé à la circulation des cyclistes. Je pourrais donc croiser des vélos venant en sens inverse, mais pas de voiture.</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>video_9/v9q10.jpg</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
         <is>
           <t>image</t>
         </is>

</xml_diff>

<commit_message>
refactor(content): add alcool-stupéfiants theme
Regroup the 6 alcohol/drug questions (limits, effects, elimination,
alcoolémie peak) under a dedicated theme instead of scattering them
across documents/assurance-constat/premiers-secours.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/questions.xlsx
+++ b/backend/data/questions.xlsx
@@ -1178,7 +1178,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>premiers-secours</t>
+          <t>alcool-stupéfiants</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>premiers-secours</t>
+          <t>alcool-stupéfiants</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>documents</t>
+          <t>alcool-stupéfiants</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>documents</t>
+          <t>alcool-stupéfiants</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>assurance-constat</t>
+          <t>alcool-stupéfiants</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>premiers-secours</t>
+          <t>alcool-stupéfiants</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">

</xml_diff>